<commit_message>
Revert status to Failed and optimize map card query with iwloc=addr
</commit_message>
<xml_diff>
--- a/src/data/uploads/test1___c0b58141-6531-45ab-be99-faa69ecb72a1.xlsx
+++ b/src/data/uploads/test1___c0b58141-6531-45ab-be99-faa69ecb72a1.xlsx
@@ -485,7 +485,7 @@
         <v>Yes</v>
       </c>
       <c r="F4" t="str">
-        <v>Uncalled</v>
+        <v>Failed to Call</v>
       </c>
       <c r="G4" t="str">
         <v/>
@@ -508,7 +508,7 @@
         <v>Yes</v>
       </c>
       <c r="F5" t="str">
-        <v>Uncalled</v>
+        <v>Failed to Call</v>
       </c>
       <c r="G5" t="str">
         <v/>
@@ -531,7 +531,7 @@
         <v>Yes</v>
       </c>
       <c r="F6" t="str">
-        <v>Uncalled</v>
+        <v>Failed to Call</v>
       </c>
       <c r="G6" t="str">
         <v/>

</xml_diff>